<commit_message>
Fix error in for some student not study enough 128 credits
</commit_message>
<xml_diff>
--- a/synthetic_data/academic_validation_report.xlsx
+++ b/synthetic_data/academic_validation_report.xlsx
@@ -1423,10 +1423,10 @@
         <v>894</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.5123042505592841</v>
+        <v>0.5044742729306487</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -1442,10 +1442,10 @@
         <v>912</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>467</v>
+        <v>456</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>0.5120614035087719</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -1461,10 +1461,10 @@
         <v>932</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>472</v>
+        <v>458</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.5064377682403434</v>
+        <v>0.4914163090128755</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -1543,28 +1543,28 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>6.809369562881911</v>
+        <v>6.831902738292663</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>2.575255655097496</v>
+        <v>2.590941389900695</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>0.05084745762711865</v>
+        <v>0.04601990049751244</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>0.1682808716707022</v>
+        <v>0.1716417910447761</v>
       </c>
       <c r="G14" s="16" t="n">
-        <v>0.1937046004842615</v>
+        <v>0.1965174129353234</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>0.1343825665859564</v>
+        <v>0.1368159203980099</v>
       </c>
       <c r="I14" s="16" t="n">
-        <v>0.2421307506053269</v>
+        <v>0.2475124378109453</v>
       </c>
       <c r="J14" s="16" t="n">
-        <v>0.2094430992736077</v>
+        <v>0.1965174129353234</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -1577,28 +1577,28 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>6.644755088537025</v>
+        <v>6.682858470129588</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>2.469338147191233</v>
+        <v>2.495151015185805</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>0.04522613065326633</v>
+        <v>0.04166666666666666</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>0.07412060301507538</v>
+        <v>0.08333333333333333</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.2964824120603015</v>
+        <v>0.2994791666666667</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>0.0414572864321608</v>
+        <v>0.03515625</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>0.2964824120603015</v>
+        <v>0.3138020833333333</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.2462311557788945</v>
+        <v>0.2239583333333333</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -1611,28 +1611,28 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>6.964651602840553</v>
+        <v>6.949426835737116</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>2.682175589763646</v>
+        <v>2.673946834797088</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>0.05709624796084829</v>
+        <v>0.04568527918781726</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>0.2822185970636215</v>
+        <v>0.2910321489001692</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>0.07504078303425775</v>
+        <v>0.06937394247038917</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>0.2316476345840131</v>
+        <v>0.245346869712352</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>0.1435562805872757</v>
+        <v>0.1404399323181049</v>
       </c>
       <c r="J16" s="16" t="n">
-        <v>0.2104404567699837</v>
+        <v>0.2081218274111675</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
@@ -1746,10 +1746,10 @@
         <v>466</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.5128755364806867</v>
+        <v>0.5042918454935622</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -1765,10 +1765,10 @@
         <v>464</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>0.4719827586206897</v>
+        <v>0.4698275862068966</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -1784,10 +1784,10 @@
         <v>469</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.4733475479744136</v>
+        <v>0.4584221748400853</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>7.294876943096911</v>
+        <v>7.267342395587077</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>2.886249584205783</v>
+        <v>2.871325847123719</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>0.1415525114155251</v>
+        <v>0.1229314420803782</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>0.2237442922374429</v>
+        <v>0.2293144208037825</v>
       </c>
       <c r="G14" s="16" t="n">
-        <v>0.2511415525114155</v>
+        <v>0.2600472813238771</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>0.0958904109589041</v>
+        <v>0.09692671394799054</v>
       </c>
       <c r="I14" s="16" t="n">
-        <v>0.1689497716894977</v>
+        <v>0.1773049645390071</v>
       </c>
       <c r="J14" s="16" t="n">
-        <v>0.1187214611872146</v>
+        <v>0.1134751773049645</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -1900,28 +1900,28 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>7.075305877994856</v>
+        <v>7.0474375</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>2.750290344248728</v>
+        <v>2.7328125</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>0.1146341463414634</v>
+        <v>0.0975</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>0.08292682926829269</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.3780487804878049</v>
+        <v>0.395</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>0.05609756097560976</v>
+        <v>0.0575</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>0.2268292682926829</v>
+        <v>0.235</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.1341463414634146</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -1934,28 +1934,28 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>7.544734575124126</v>
+        <v>7.486681084198384</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>3.044456690174251</v>
+        <v>3.009991349480969</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>0.1628664495114006</v>
+        <v>0.1384083044982699</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>0.3615635179153094</v>
+        <v>0.384083044982699</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>0.1433224755700326</v>
+        <v>0.1314878892733564</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>0.1433224755700326</v>
+        <v>0.1557093425605536</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>0.08794788273615635</v>
+        <v>0.08650519031141868</v>
       </c>
       <c r="J16" s="16" t="n">
-        <v>0.09771986970684039</v>
+        <v>0.1038062283737024</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
@@ -2107,10 +2107,10 @@
         <v>157</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.5031847133757962</v>
+        <v>0.464968152866242</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -2189,28 +2189,28 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>7.716682074223738</v>
+        <v>7.699739583333333</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>3.157480023271047</v>
+        <v>3.147493489583333</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.2578125</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>0.2230769230769231</v>
+        <v>0.234375</v>
       </c>
       <c r="G14" s="16" t="n">
-        <v>0.2923076923076923</v>
+        <v>0.2890625</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>0.06153846153846154</v>
+        <v>0.0625</v>
       </c>
       <c r="I14" s="16" t="n">
-        <v>0.1</v>
+        <v>0.1015625</v>
       </c>
       <c r="J14" s="16" t="n">
-        <v>0.05384615384615385</v>
+        <v>0.0546875</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -2223,28 +2223,28 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>7.745482833825806</v>
+        <v>7.688169191919192</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>3.183755100605037</v>
+        <v>3.15123106060606</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>0.2826086956521739</v>
+        <v>0.25</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>0.08695652173913043</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.4855072463768116</v>
+        <v>0.5151515151515151</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>0.05072463768115942</v>
+        <v>0.04545454545454546</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>0.08695652173913043</v>
+        <v>0.09848484848484848</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.007246376811594203</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -2257,28 +2257,28 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>7.815767314476835</v>
+        <v>7.752718855218855</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>3.208081915316705</v>
+        <v>3.177609427609428</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>0.2300884955752212</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>0.4070796460176991</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>0.1327433628318584</v>
+        <v>0.1313131313131313</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>0.1150442477876106</v>
+        <v>0.1313131313131313</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>0.07079646017699115</v>
+        <v>0.0707070707070707</v>
       </c>
       <c r="J16" s="16" t="n">
-        <v>0.04424778761061947</v>
+        <v>0.04040404040404041</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">

</xml_diff>

<commit_message>
Update data more realistic in clc and advanced
</commit_message>
<xml_diff>
--- a/synthetic_data/academic_validation_report.xlsx
+++ b/synthetic_data/academic_validation_report.xlsx
@@ -979,7 +979,7 @@
       <row>18</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="4140000"/>
+    <ext cx="7920000" cy="3888000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1006,7 +1006,7 @@
       <row>18</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="4140000"/>
+    <ext cx="7920000" cy="3888000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1033,7 +1033,7 @@
       <row>18</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="4140000"/>
+    <ext cx="7920000" cy="3888000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1372,7 +1372,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ĐẶC TRƯNG 1: TIẾN ĐỘ TỐT NGHIỆP VÀ PHÂN BỐ ĐIỂM SỐ SINH VIÊN (K20, K21, K22) | Quy mô: 6,703 SV (60.7% toàn trường)</t>
+          <t>BÁO CÁO HỌC VỤ: TIẾN ĐỘ TỐT NGHIỆP, XẾP LOẠI ĐIỂM &amp; TỶ LỆ BỎ HỌC (K20 - K26) | Quy mô: 6,703 SV (60.7% toàn trường)</t>
         </is>
       </c>
     </row>
@@ -1423,10 +1423,10 @@
         <v>894</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>451</v>
+        <v>506</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.5044742729306487</v>
+        <v>0.5659955257270693</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -1442,10 +1442,10 @@
         <v>912</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>456</v>
+        <v>482</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>0.5</v>
+        <v>0.5285087719298246</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -1461,10 +1461,10 @@
         <v>932</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>458</v>
+        <v>514</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.4914163090128755</v>
+        <v>0.5515021459227468</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -1543,28 +1543,28 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>6.831902738292663</v>
+        <v>6.945755988792428</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>2.590941389900695</v>
+        <v>2.670855254832579</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>0.04601990049751244</v>
+        <v>0.049338146811071</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>0.1716417910447761</v>
+        <v>0.1660649819494585</v>
       </c>
       <c r="G14" s="16" t="n">
-        <v>0.1965174129353234</v>
+        <v>0.2093862815884477</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>0.1368159203980099</v>
+        <v>0.1335740072202166</v>
       </c>
       <c r="I14" s="16" t="n">
-        <v>0.2475124378109453</v>
+        <v>0.4416365824308063</v>
       </c>
       <c r="J14" s="16" t="n">
-        <v>0.1965174129353234</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -1577,28 +1577,28 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>6.682858470129588</v>
+        <v>6.87467448730367</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>2.495151015185805</v>
+        <v>2.626924075896763</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.04724409448818898</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.08530183727034121</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.2994791666666667</v>
+        <v>0.3228346456692913</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>0.03515625</v>
+        <v>0.03805774278215223</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>0.3138020833333333</v>
+        <v>0.5065616797900262</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.2239583333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -1611,28 +1611,28 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>6.949426835737116</v>
+        <v>7.150501072563236</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>2.673946834797088</v>
+        <v>2.807529907570962</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>0.04568527918781726</v>
+        <v>0.05255023183925812</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>0.2910321489001692</v>
+        <v>0.3137557959814529</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>0.06937394247038917</v>
+        <v>0.08964451313755796</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>0.245346869712352</v>
+        <v>0.2519319938176198</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>0.1404399323181049</v>
+        <v>0.2921174652241113</v>
       </c>
       <c r="J16" s="16" t="n">
-        <v>0.2081218274111675</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
@@ -1642,8 +1642,183 @@
         </is>
       </c>
     </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>III. BẢNG 3: TỶ LỆ BỎ HỌC TỪNG KHÓA (KHÓA K20 ĐẾN K26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Khóa học</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Sĩ số tuyển sinh (SV)</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Sinh viên bỏ học (SV)</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Tỷ lệ bỏ học (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K20</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>894</v>
+      </c>
+      <c r="D46" s="12" t="n">
+        <v>63</v>
+      </c>
+      <c r="E46" s="13" t="n">
+        <v>0.07046979865771812</v>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Khóa K21</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="n">
+        <v>912</v>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>0.01096491228070175</v>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K22</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="n">
+        <v>932</v>
+      </c>
+      <c r="D48" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E48" s="13" t="n">
+        <v>0.01072961373390558</v>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Khóa K23</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="n">
+        <v>986</v>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>0.01115618661257606</v>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K24</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="n">
+        <v>960</v>
+      </c>
+      <c r="D50" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="E50" s="13" t="n">
+        <v>0.015625</v>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Khóa K25</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="n">
+        <v>978</v>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>0.01431492842535787</v>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K26</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="n">
+        <v>1041</v>
+      </c>
+      <c r="D52" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E52" s="13" t="n">
+        <v>0.01536983669548511</v>
+      </c>
+    </row>
+    <row r="53" ht="24" customHeight="1">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>💡 Cách tính: Tỷ lệ bỏ học = Số sinh viên bỏ học (dropout = True) / Tổng sĩ số sinh viên của khóa.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
+    <mergeCell ref="A53:E53"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A17:J17"/>
     <mergeCell ref="A10:E10"/>
@@ -1651,6 +1826,7 @@
     <mergeCell ref="A12:J12"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A44:E44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1663,7 +1839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1695,7 +1871,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ĐẶC TRƯNG 1: TIẾN ĐỘ TỐT NGHIỆP VÀ PHÂN BỐ ĐIỂM SỐ SINH VIÊN (K20, K21, K22) | Quy mô: 3,277 SV (29.7% toàn trường)</t>
+          <t>BÁO CÁO HỌC VỤ: TIẾN ĐỘ TỐT NGHIỆP, XẾP LOẠI ĐIỂM &amp; TỶ LỆ BỎ HỌC (K20 - K26) | Quy mô: 3,277 SV (29.7% toàn trường)</t>
         </is>
       </c>
     </row>
@@ -1746,10 +1922,10 @@
         <v>466</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>235</v>
+        <v>403</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.5042918454935622</v>
+        <v>0.8648068669527897</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -1765,10 +1941,10 @@
         <v>464</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>218</v>
+        <v>403</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>0.4698275862068966</v>
+        <v>0.8685344827586207</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -1784,10 +1960,10 @@
         <v>469</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>215</v>
+        <v>401</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.4584221748400853</v>
+        <v>0.8550106609808102</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -1866,28 +2042,28 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>7.267342395587077</v>
+        <v>7.320655430711611</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>2.871325847123719</v>
+        <v>2.909794007490636</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>0.1229314420803782</v>
+        <v>0.1213483146067416</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>0.2293144208037825</v>
+        <v>0.2247191011235955</v>
       </c>
       <c r="G14" s="16" t="n">
-        <v>0.2600472813238771</v>
+        <v>0.2651685393258427</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>0.09692671394799054</v>
+        <v>0.09662921348314607</v>
       </c>
       <c r="I14" s="16" t="n">
-        <v>0.1773049645390071</v>
+        <v>0.2921348314606741</v>
       </c>
       <c r="J14" s="16" t="n">
-        <v>0.1134751773049645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -1900,28 +2076,28 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>7.0474375</v>
+        <v>7.166383181126332</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>2.7328125</v>
+        <v>2.815848554033486</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>0.0975</v>
+        <v>0.1073059360730594</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.0776255707762557</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.395</v>
+        <v>0.4200913242009132</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>0.0575</v>
+        <v>0.05707762557077625</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>0.235</v>
+        <v>0.3378995433789954</v>
       </c>
       <c r="J15" s="18" t="n">
-        <v>0.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
@@ -1934,28 +2110,28 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>7.486681084198384</v>
+        <v>7.576694577352472</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>3.009991349480969</v>
+        <v>3.06966706539075</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>0.1384083044982699</v>
+        <v>0.1578947368421053</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>0.384083044982699</v>
+        <v>0.3564593301435406</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>0.1314878892733564</v>
+        <v>0.1626794258373206</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>0.1557093425605536</v>
+        <v>0.1435406698564593</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>0.08650519031141868</v>
+        <v>0.1794258373205742</v>
       </c>
       <c r="J16" s="16" t="n">
-        <v>0.1038062283737024</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
@@ -1965,8 +2141,183 @@
         </is>
       </c>
     </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>III. BẢNG 3: TỶ LỆ BỎ HỌC TỪNG KHÓA (KHÓA K20 ĐẾN K26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Khóa học</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Sĩ số tuyển sinh (SV)</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Sinh viên bỏ học (SV)</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Tỷ lệ bỏ học (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K20</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>466</v>
+      </c>
+      <c r="D46" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="E46" s="13" t="n">
+        <v>0.04506437768240344</v>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Khóa K21</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="n">
+        <v>464</v>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K22</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="n">
+        <v>469</v>
+      </c>
+      <c r="D48" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Khóa K23</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="n">
+        <v>435</v>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K24</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="n">
+        <v>476</v>
+      </c>
+      <c r="D50" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Khóa K25</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="n">
+        <v>491</v>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K26</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="n">
+        <v>476</v>
+      </c>
+      <c r="D52" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" ht="24" customHeight="1">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>💡 Cách tính: Tỷ lệ bỏ học = Số sinh viên bỏ học (dropout = True) / Tổng sĩ số sinh viên của khóa.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
+    <mergeCell ref="A53:E53"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A17:J17"/>
     <mergeCell ref="A10:E10"/>
@@ -1974,6 +2325,7 @@
     <mergeCell ref="A12:J12"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A44:E44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1986,7 +2338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2018,7 +2370,7 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ĐẶC TRƯNG 1: TIẾN ĐỘ TỐT NGHIỆP VÀ PHÂN BỐ ĐIỂM SỐ SINH VIÊN (K20, K21, K22) | Quy mô: 1,071 SV (9.7% toàn trường)</t>
+          <t>BÁO CÁO HỌC VỤ: TIẾN ĐỘ TỐT NGHIỆP, XẾP LOẠI ĐIỂM &amp; TỶ LỆ BỎ HỌC (K20 - K26) | Quy mô: 1,071 SV (9.7% toàn trường)</t>
         </is>
       </c>
     </row>
@@ -2069,10 +2421,10 @@
         <v>140</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>66</v>
+        <v>134</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.4714285714285714</v>
+        <v>0.9571428571428572</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -2088,10 +2440,10 @@
         <v>153</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>82</v>
+        <v>147</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>0.5359477124183006</v>
+        <v>0.9607843137254902</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -2107,10 +2459,10 @@
         <v>157</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>73</v>
+        <v>136</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.464968152866242</v>
+        <v>0.8662420382165605</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -2189,28 +2541,28 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>7.699739583333333</v>
+        <v>7.745328467153286</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>3.147493489583333</v>
+        <v>3.179470802919708</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>0.2578125</v>
+        <v>0.2554744525547445</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>0.234375</v>
+        <v>0.2408759124087591</v>
       </c>
       <c r="G14" s="16" t="n">
-        <v>0.2890625</v>
+        <v>0.2992700729927008</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>0.0625</v>
+        <v>0.06569343065693431</v>
       </c>
       <c r="I14" s="16" t="n">
-        <v>0.1015625</v>
+        <v>0.1386861313868613</v>
       </c>
       <c r="J14" s="16" t="n">
-        <v>0.0546875</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
@@ -2223,25 +2575,25 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>7.688169191919192</v>
+        <v>7.66858843537415</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>3.15123106060606</v>
+        <v>3.139569160997732</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>0.25</v>
+        <v>0.2380952380952381</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.5151515151515151</v>
+        <v>0.5102040816326531</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>0.04545454545454546</v>
+        <v>0.06802721088435375</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>0.09848484848484848</v>
+        <v>0.08843537414965986</v>
       </c>
       <c r="J15" s="18" t="n">
         <v>0</v>
@@ -2257,28 +2609,28 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>7.752718855218855</v>
+        <v>7.826038647342995</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>3.177609427609428</v>
+        <v>3.223037439613526</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.1884057971014493</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.4565217391304348</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>0.1313131313131313</v>
+        <v>0.1594202898550725</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>0.1313131313131313</v>
+        <v>0.1014492753623188</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>0.0707070707070707</v>
+        <v>0.09420289855072464</v>
       </c>
       <c r="J16" s="16" t="n">
-        <v>0.04040404040404041</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
@@ -2288,8 +2640,183 @@
         </is>
       </c>
     </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>III. BẢNG 3: TỶ LỆ BỎ HỌC TỪNG KHÓA (KHÓA K20 ĐẾN K26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Khóa học</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Sĩ số tuyển sinh (SV)</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Sinh viên bỏ học (SV)</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Tỷ lệ bỏ học (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K20</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>140</v>
+      </c>
+      <c r="D46" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" s="13" t="n">
+        <v>0.02142857142857143</v>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Khóa K21</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="n">
+        <v>153</v>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K22</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="n">
+        <v>157</v>
+      </c>
+      <c r="D48" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Khóa K23</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="n">
+        <v>157</v>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K24</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="n">
+        <v>162</v>
+      </c>
+      <c r="D50" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Khóa K25</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="n">
+        <v>158</v>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>Khóa K26</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="n">
+        <v>144</v>
+      </c>
+      <c r="D52" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" ht="24" customHeight="1">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>💡 Cách tính: Tỷ lệ bỏ học = Số sinh viên bỏ học (dropout = True) / Tổng sĩ số sinh viên của khóa.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
+    <mergeCell ref="A53:E53"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A17:J17"/>
     <mergeCell ref="A10:E10"/>
@@ -2297,6 +2824,7 @@
     <mergeCell ref="A12:J12"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A44:E44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Update credits each term for early graduated
</commit_message>
<xml_diff>
--- a/synthetic_data/academic_validation_report.xlsx
+++ b/synthetic_data/academic_validation_report.xlsx
@@ -1423,10 +1423,10 @@
         <v>894</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>506</v>
+        <v>497</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.5659955257270693</v>
+        <v>0.5559284116331096</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -1442,10 +1442,10 @@
         <v>912</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>0.5285087719298246</v>
+        <v>0.5274122807017544</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -1461,10 +1461,10 @@
         <v>932</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.5515021459227468</v>
+        <v>0.5472103004291845</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -1543,25 +1543,25 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>6.945755988792428</v>
+        <v>6.943340416523752</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>2.670855254832579</v>
+        <v>2.669240240739153</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>0.049338146811071</v>
+        <v>0.04921968787515006</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>0.1660649819494585</v>
+        <v>0.1656662665066026</v>
       </c>
       <c r="G14" s="16" t="n">
-        <v>0.2093862815884477</v>
+        <v>0.2088835534213686</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>0.1335740072202166</v>
+        <v>0.1332533013205282</v>
       </c>
       <c r="I14" s="16" t="n">
-        <v>0.4416365824308063</v>
+        <v>0.4429771908763505</v>
       </c>
       <c r="J14" s="16" t="n">
         <v>0</v>
@@ -1577,25 +1577,25 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>6.87467448730367</v>
+        <v>6.874925269330246</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>2.626924075896763</v>
+        <v>2.626986408339069</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>0.04724409448818898</v>
+        <v>0.04730617608409987</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>0.08530183727034121</v>
+        <v>0.08541392904073587</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.3228346456692913</v>
+        <v>0.3232588699080158</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>0.03805774278215223</v>
+        <v>0.03810775295663601</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>0.5065616797900262</v>
+        <v>0.5059132720105125</v>
       </c>
       <c r="J15" s="18" t="n">
         <v>0</v>
@@ -1611,25 +1611,25 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>7.150501072563236</v>
+        <v>7.155333900996993</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>2.807529907570962</v>
+        <v>2.810884912162329</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>0.05255023183925812</v>
+        <v>0.05279503105590062</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>0.3137557959814529</v>
+        <v>0.3152173913043478</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>0.08964451313755796</v>
+        <v>0.09006211180124224</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>0.2519319938176198</v>
+        <v>0.2531055900621118</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>0.2921174652241113</v>
+        <v>0.2888198757763975</v>
       </c>
       <c r="J16" s="16" t="n">
         <v>0</v>
@@ -1689,10 +1689,10 @@
         <v>894</v>
       </c>
       <c r="D46" s="12" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E46" s="13" t="n">
-        <v>0.07046979865771812</v>
+        <v>0.06823266219239374</v>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
@@ -1922,10 +1922,10 @@
         <v>466</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.8648068669527897</v>
+        <v>0.8540772532188842</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -1941,10 +1941,10 @@
         <v>464</v>
       </c>
       <c r="D8" s="12" t="n">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>0.8685344827586207</v>
+        <v>0.8642241379310345</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -1960,10 +1960,10 @@
         <v>469</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.8550106609808102</v>
+        <v>0.8507462686567164</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
@@ -2042,10 +2042,10 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>7.320655430711611</v>
+        <v>7.321142322097379</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>2.909794007490636</v>
+        <v>2.909971910112359</v>
       </c>
       <c r="E14" s="16" t="n">
         <v>0.1213483146067416</v>
@@ -2076,25 +2076,25 @@
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>7.166383181126332</v>
+        <v>7.17365634556575</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>2.815848554033486</v>
+        <v>2.820422400611621</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>0.1073059360730594</v>
+        <v>0.1077981651376147</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>0.0776255707762557</v>
+        <v>0.07798165137614679</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>0.4200913242009132</v>
+        <v>0.4220183486238532</v>
       </c>
       <c r="H15" s="18" t="n">
-        <v>0.05707762557077625</v>
+        <v>0.05733944954128441</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>0.3378995433789954</v>
+        <v>0.3348623853211009</v>
       </c>
       <c r="J15" s="18" t="n">
         <v>0</v>
@@ -2110,25 +2110,25 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>7.576694577352472</v>
+        <v>7.587451807228915</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>3.06966706539075</v>
+        <v>3.07656626506024</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>0.1578947368421053</v>
+        <v>0.1590361445783132</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>0.3564593301435406</v>
+        <v>0.3590361445783132</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>0.1626794258373206</v>
+        <v>0.163855421686747</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>0.1435406698564593</v>
+        <v>0.144578313253012</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>0.1794258373205742</v>
+        <v>0.1734939759036145</v>
       </c>
       <c r="J16" s="16" t="n">
         <v>0</v>
@@ -2541,10 +2541,10 @@
         </is>
       </c>
       <c r="C14" s="15" t="n">
-        <v>7.745328467153286</v>
+        <v>7.744701946472021</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>3.179470802919708</v>
+        <v>3.178923357664234</v>
       </c>
       <c r="E14" s="16" t="n">
         <v>0.2554744525547445</v>
@@ -2609,25 +2609,25 @@
         </is>
       </c>
       <c r="C16" s="15" t="n">
-        <v>7.826038647342995</v>
+        <v>7.839422141119219</v>
       </c>
       <c r="D16" s="15" t="n">
-        <v>3.223037439613526</v>
+        <v>3.231660583941605</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>0.1884057971014493</v>
+        <v>0.1897810218978102</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>0.4565217391304348</v>
+        <v>0.4598540145985401</v>
       </c>
       <c r="G16" s="16" t="n">
-        <v>0.1594202898550725</v>
+        <v>0.1605839416058394</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>0.1014492753623188</v>
+        <v>0.1021897810218978</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>0.09420289855072464</v>
+        <v>0.08759124087591241</v>
       </c>
       <c r="J16" s="16" t="n">
         <v>0</v>

</xml_diff>